<commit_message>
Add parallel execution support and update documentation
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnandaroopMaitra(G10\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnandaroopMaitra(G10\IdeaProjects\SeleniumJavaFramework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5F674E-4A65-4C67-97BB-D742B27D6A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E37635-4C07-4319-8E09-26AC0AC613BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
   <si>
     <t>Username</t>
   </si>
@@ -58,6 +58,18 @@
   </si>
   <si>
     <t>abc123</t>
+  </si>
+  <si>
+    <t>wrong123</t>
+  </si>
+  <si>
+    <t>Wrong</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>User123</t>
   </si>
 </sst>
 </file>
@@ -389,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.26953125" customWidth="1"/>
@@ -397,7 +409,7 @@
     <col min="3" max="3" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -408,7 +420,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -430,7 +442,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -449,6 +461,50 @@
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>